<commit_message>
allow kevin token update and keep Excel hours
</commit_message>
<xml_diff>
--- a/data/horaires_complet.xlsx
+++ b/data/horaires_complet.xlsx
@@ -74,7 +74,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -110,11 +110,77 @@
         <color rgb="00DDDDDD"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00AAAAAA"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00AAAAAA"/>
+      </left>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00AAAAAA"/>
+      </left>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -137,6 +203,8 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -563,38 +631,51 @@
           <t>Lundi</t>
         </is>
       </c>
+      <c r="H1" s="8" t="n"/>
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Mardi</t>
         </is>
       </c>
+      <c r="J1" s="8" t="n"/>
       <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Mercredi</t>
         </is>
       </c>
+      <c r="L1" s="8" t="n"/>
       <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Jeudi</t>
         </is>
       </c>
+      <c r="N1" s="8" t="n"/>
       <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Vendredi</t>
         </is>
       </c>
+      <c r="P1" s="8" t="n"/>
       <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Samedi</t>
         </is>
       </c>
+      <c r="R1" s="8" t="n"/>
       <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Dimanche</t>
         </is>
       </c>
+      <c r="T1" s="8" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="9" t="n"/>
+      <c r="B2" s="9" t="n"/>
+      <c r="C2" s="9" t="n"/>
+      <c r="D2" s="9" t="n"/>
+      <c r="E2" s="9" t="n"/>
+      <c r="F2" s="9" t="n"/>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Matin</t>
@@ -22177,46 +22258,46 @@
       </c>
       <c r="G282" s="6" t="inlineStr">
         <is>
-          <t>Fermé</t>
-        </is>
-      </c>
-      <c r="H282" s="6" t="inlineStr"/>
+          <t>07:00 - 19:30</t>
+        </is>
+      </c>
+      <c r="H282" s="6" t="n"/>
       <c r="I282" s="6" t="inlineStr">
         <is>
-          <t>Fermé</t>
-        </is>
-      </c>
-      <c r="J282" s="6" t="inlineStr"/>
+          <t>07:00 - 19:30</t>
+        </is>
+      </c>
+      <c r="J282" s="6" t="n"/>
       <c r="K282" s="6" t="inlineStr">
         <is>
-          <t>Fermé</t>
-        </is>
-      </c>
-      <c r="L282" s="6" t="inlineStr"/>
+          <t>07:00 - 19:30</t>
+        </is>
+      </c>
+      <c r="L282" s="6" t="n"/>
       <c r="M282" s="6" t="inlineStr">
         <is>
-          <t>Fermé</t>
-        </is>
-      </c>
-      <c r="N282" s="6" t="inlineStr"/>
+          <t>07:00 - 19:30</t>
+        </is>
+      </c>
+      <c r="N282" s="6" t="n"/>
       <c r="O282" s="6" t="inlineStr">
         <is>
-          <t>Fermé</t>
-        </is>
-      </c>
-      <c r="P282" s="6" t="inlineStr"/>
+          <t>07:00 - 19:30</t>
+        </is>
+      </c>
+      <c r="P282" s="6" t="n"/>
       <c r="Q282" s="6" t="inlineStr">
         <is>
-          <t>Fermé</t>
-        </is>
-      </c>
-      <c r="R282" s="6" t="inlineStr"/>
+          <t>08:30 - 19:30</t>
+        </is>
+      </c>
+      <c r="R282" s="6" t="n"/>
       <c r="S282" s="6" t="inlineStr">
         <is>
-          <t>Fermé</t>
-        </is>
-      </c>
-      <c r="T282" s="6" t="inlineStr"/>
+          <t>08:30 - 17:30</t>
+        </is>
+      </c>
+      <c r="T282" s="6" t="n"/>
     </row>
     <row r="283" ht="15" customHeight="1">
       <c r="A283" s="4" t="inlineStr">
@@ -27663,46 +27744,46 @@
       </c>
       <c r="G353" s="4" t="inlineStr">
         <is>
-          <t>00:00 - 23:59</t>
-        </is>
-      </c>
-      <c r="H353" s="4" t="inlineStr"/>
+          <t>09:00 - 22:00</t>
+        </is>
+      </c>
+      <c r="H353" s="4" t="n"/>
       <c r="I353" s="4" t="inlineStr">
         <is>
-          <t>00:00 - 23:59</t>
-        </is>
-      </c>
-      <c r="J353" s="4" t="inlineStr"/>
+          <t>09:00 - 22:00</t>
+        </is>
+      </c>
+      <c r="J353" s="4" t="n"/>
       <c r="K353" s="4" t="inlineStr">
         <is>
-          <t>00:00 - 23:59</t>
-        </is>
-      </c>
-      <c r="L353" s="4" t="inlineStr"/>
+          <t>09:00 - 22:00</t>
+        </is>
+      </c>
+      <c r="L353" s="4" t="n"/>
       <c r="M353" s="4" t="inlineStr">
         <is>
-          <t>00:00 - 23:59</t>
-        </is>
-      </c>
-      <c r="N353" s="4" t="inlineStr"/>
+          <t>09:00 - 22:00</t>
+        </is>
+      </c>
+      <c r="N353" s="4" t="n"/>
       <c r="O353" s="4" t="inlineStr">
         <is>
-          <t>00:00 - 23:59</t>
-        </is>
-      </c>
-      <c r="P353" s="4" t="inlineStr"/>
+          <t>09:00 - 22:00</t>
+        </is>
+      </c>
+      <c r="P353" s="4" t="n"/>
       <c r="Q353" s="4" t="inlineStr">
         <is>
-          <t>00:00 - 23:59</t>
-        </is>
-      </c>
-      <c r="R353" s="4" t="inlineStr"/>
+          <t>09:00 - 22:00</t>
+        </is>
+      </c>
+      <c r="R353" s="4" t="n"/>
       <c r="S353" s="4" t="inlineStr">
         <is>
-          <t>00:00 - 23:59</t>
-        </is>
-      </c>
-      <c r="T353" s="4" t="inlineStr"/>
+          <t>09:00 - 22:00</t>
+        </is>
+      </c>
+      <c r="T353" s="4" t="n"/>
     </row>
     <row r="354" ht="15" customHeight="1">
       <c r="A354" s="6" t="inlineStr">

</xml_diff>